<commit_message>
Code.gs v1.6 / page v1.4.3: EcoOils (Project), EcoOils (Operations) and Other applicants
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019wC6HTWyTgwVhiZHSRJnLE
</commit_message>
<xml_diff>
--- a/templates/PTW_Registry_Template_ENTRY.xlsx
+++ b/templates/PTW_Registry_Template_ENTRY.xlsx
@@ -1126,32 +1126,11 @@
           <t>TYPE OF WORK  /  JENIS PEKERJAAN  (Y = yes)</t>
         </is>
       </c>
-      <c r="K2" s="9" t="n"/>
-      <c r="L2" s="9" t="n"/>
-      <c r="M2" s="9" t="n"/>
-      <c r="N2" s="9" t="n"/>
-      <c r="O2" s="9" t="n"/>
-      <c r="P2" s="9" t="n"/>
-      <c r="Q2" s="9" t="n"/>
-      <c r="R2" s="9" t="n"/>
-      <c r="S2" s="9" t="n"/>
-      <c r="T2" s="9" t="n"/>
       <c r="V2" s="8" t="inlineStr">
         <is>
           <t>SUPPORTING DOCUMENTS  /  DOKUMEN PENDUKUNG  (Y = attached)</t>
         </is>
       </c>
-      <c r="W2" s="9" t="n"/>
-      <c r="X2" s="9" t="n"/>
-      <c r="Y2" s="9" t="n"/>
-      <c r="Z2" s="9" t="n"/>
-      <c r="AA2" s="9" t="n"/>
-      <c r="AB2" s="9" t="n"/>
-      <c r="AC2" s="9" t="n"/>
-      <c r="AD2" s="9" t="n"/>
-      <c r="AE2" s="9" t="n"/>
-      <c r="AF2" s="9" t="n"/>
-      <c r="AG2" s="9" t="n"/>
     </row>
     <row r="3" ht="150" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -12155,8 +12134,8 @@
     <mergeCell ref="V2:AG2"/>
   </mergeCells>
   <dataValidations count="34">
-    <dataValidation sqref="B5:B204" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from list" error="Please choose a value from the dropdown. / Pilih dari daftar." type="list" errorStyle="stop">
-      <formula1>=Lists!$E$2:$E$5</formula1>
+    <dataValidation sqref="B5:B204" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Applicant company" error="Pick from the list, or type: Other: &lt;company name&gt; / Pilih dari daftar, atau ketik: Other: &lt;nama perusahaan&gt;" promptTitle="Applicant company" prompt="GSB, WEN, KKS, PBS, EcoOils (Project), EcoOils (Operations), or type  Other: &lt;company name&gt;" type="list" errorStyle="warning">
+      <formula1>=Lists!$E$2:$E$7</formula1>
     </dataValidation>
     <dataValidation sqref="D5:D204" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the list" error="Not on the list. Choose Yes to keep it as a new entry. / Tidak ada di daftar. Pilih Yes untuk tetap memakainya." type="list" errorStyle="warning">
       <formula1>=Lists!$G$2:$G$19</formula1>
@@ -15082,8 +15061,8 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0" password="E84A"/>
   <dataValidations count="6">
-    <dataValidation sqref="B5:B204" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from list" error="Please choose a value from the dropdown. / Pilih dari daftar." type="list" errorStyle="stop">
-      <formula1>=Lists!$E$2:$E$5</formula1>
+    <dataValidation sqref="B5:B204" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Applicant company" error="Pick from the list, or type: Other: &lt;company name&gt; / Pilih dari daftar, atau ketik: Other: &lt;nama perusahaan&gt;" promptTitle="Applicant company" prompt="GSB, WEN, KKS, PBS, EcoOils (Project), EcoOils (Operations), or type  Other: &lt;company name&gt;" type="list" errorStyle="warning">
+      <formula1>=Lists!$E$2:$E$7</formula1>
     </dataValidation>
     <dataValidation sqref="C5:C204" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Day" error="Day must be 2 to 7. After 7 days a NEW PTW is needed. / Hari harus 2-7. Setelah 7 hari wajib PTW baru." type="list" errorStyle="stop">
       <formula1>=Lists!$F$2:$F$7</formula1>
@@ -17055,8 +17034,8 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0" password="E84A"/>
   <dataValidations count="4">
-    <dataValidation sqref="B5:B204" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from list" error="Please choose a value from the dropdown. / Pilih dari daftar." type="list" errorStyle="stop">
-      <formula1>=Lists!$E$2:$E$5</formula1>
+    <dataValidation sqref="B5:B204" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Applicant company" error="Pick from the list, or type: Other: &lt;company name&gt; / Pilih dari daftar, atau ketik: Other: &lt;nama perusahaan&gt;" promptTitle="Applicant company" prompt="GSB, WEN, KKS, PBS, EcoOils (Project), EcoOils (Operations), or type  Other: &lt;company name&gt;" type="list" errorStyle="warning">
+      <formula1>=Lists!$E$2:$E$7</formula1>
     </dataValidation>
     <dataValidation sqref="C5:C204" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Date" error="Enter a real date, e.g. 2026-10-07. / Masukkan tanggal yang valid." type="date" errorStyle="stop" operator="between">
       <formula1>45292</formula1>
@@ -17231,6 +17210,11 @@
       </c>
     </row>
     <row r="6">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>EcoOils (Project)</t>
+        </is>
+      </c>
       <c r="F6" t="n">
         <v>6</v>
       </c>
@@ -17246,6 +17230,11 @@
       </c>
     </row>
     <row r="7">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>EcoOils (Operations)</t>
+        </is>
+      </c>
       <c r="F7" t="n">
         <v>7</v>
       </c>

</xml_diff>

<commit_message>
Code.gs v1.8 / page v1.4.5: Hot Work fire watcher, Lifting plan auto-tick, Electrical isolation plan or note
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019wC6HTWyTgwVhiZHSRJnLE
</commit_message>
<xml_diff>
--- a/templates/PTW_Registry_Template_ENTRY.xlsx
+++ b/templates/PTW_Registry_Template_ENTRY.xlsx
@@ -850,7 +850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ204"/>
+  <dimension ref="A1:AS204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -896,6 +896,8 @@
     <col width="26" customWidth="1" min="41" max="41"/>
     <col width="26" customWidth="1" min="42" max="42"/>
     <col width="14" customWidth="1" min="43" max="43"/>
+    <col width="34" customWidth="1" min="44" max="44"/>
+    <col width="34" customWidth="1" min="45" max="45"/>
   </cols>
   <sheetData>
     <row r="1" hidden="1">
@@ -1114,6 +1116,16 @@
           <t>workParty</t>
         </is>
       </c>
+      <c r="AR1" s="6" t="inlineStr">
+        <is>
+          <t>fireWatcher</t>
+        </is>
+      </c>
+      <c r="AS1" s="6" t="inlineStr">
+        <is>
+          <t>isoNote</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
@@ -1391,6 +1403,18 @@
         <is>
           <t>Work party (no. of people)
 Jumlah pekerja</t>
+        </is>
+      </c>
+      <c r="AR3" s="11" t="inlineStr">
+        <is>
+          <t>Fire Watcher name (required if Hot Work)
+Nama Fire Watcher (wajib jika Kerja Panas)</t>
+        </is>
+      </c>
+      <c r="AS3" s="11" t="inlineStr">
+        <is>
+          <t>Isolation not required – reason, by Job Coordinator (needed if Electrical and no Isolation Plan)
+Isolasi tidak diperlukan – alasan oleh Job Coordinator (wajib jika Kelistrikan tanpa Rencana Isolasi)</t>
         </is>
       </c>
     </row>
@@ -1526,6 +1550,12 @@
           <t>6</t>
         </is>
       </c>
+      <c r="AR4" s="13" t="inlineStr">
+        <is>
+          <t>Budi</t>
+        </is>
+      </c>
+      <c r="AS4" s="13" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="15" t="n"/>
@@ -1579,6 +1609,8 @@
       <c r="AO5" s="15" t="n"/>
       <c r="AP5" s="15" t="n"/>
       <c r="AQ5" s="16" t="n"/>
+      <c r="AR5" s="16" t="n"/>
+      <c r="AS5" s="16" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="n"/>
@@ -1632,6 +1664,8 @@
       <c r="AO6" s="15" t="n"/>
       <c r="AP6" s="15" t="n"/>
       <c r="AQ6" s="16" t="n"/>
+      <c r="AR6" s="16" t="n"/>
+      <c r="AS6" s="16" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="n"/>
@@ -1685,6 +1719,8 @@
       <c r="AO7" s="15" t="n"/>
       <c r="AP7" s="15" t="n"/>
       <c r="AQ7" s="16" t="n"/>
+      <c r="AR7" s="16" t="n"/>
+      <c r="AS7" s="16" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="n"/>
@@ -1738,6 +1774,8 @@
       <c r="AO8" s="15" t="n"/>
       <c r="AP8" s="15" t="n"/>
       <c r="AQ8" s="16" t="n"/>
+      <c r="AR8" s="16" t="n"/>
+      <c r="AS8" s="16" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="n"/>
@@ -1791,6 +1829,8 @@
       <c r="AO9" s="15" t="n"/>
       <c r="AP9" s="15" t="n"/>
       <c r="AQ9" s="16" t="n"/>
+      <c r="AR9" s="16" t="n"/>
+      <c r="AS9" s="16" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="15" t="n"/>
@@ -1844,6 +1884,8 @@
       <c r="AO10" s="15" t="n"/>
       <c r="AP10" s="15" t="n"/>
       <c r="AQ10" s="16" t="n"/>
+      <c r="AR10" s="16" t="n"/>
+      <c r="AS10" s="16" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="n"/>
@@ -1897,6 +1939,8 @@
       <c r="AO11" s="15" t="n"/>
       <c r="AP11" s="15" t="n"/>
       <c r="AQ11" s="16" t="n"/>
+      <c r="AR11" s="16" t="n"/>
+      <c r="AS11" s="16" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="15" t="n"/>
@@ -1950,6 +1994,8 @@
       <c r="AO12" s="15" t="n"/>
       <c r="AP12" s="15" t="n"/>
       <c r="AQ12" s="16" t="n"/>
+      <c r="AR12" s="16" t="n"/>
+      <c r="AS12" s="16" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="n"/>
@@ -2003,6 +2049,8 @@
       <c r="AO13" s="15" t="n"/>
       <c r="AP13" s="15" t="n"/>
       <c r="AQ13" s="16" t="n"/>
+      <c r="AR13" s="16" t="n"/>
+      <c r="AS13" s="16" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="n"/>
@@ -2056,6 +2104,8 @@
       <c r="AO14" s="15" t="n"/>
       <c r="AP14" s="15" t="n"/>
       <c r="AQ14" s="16" t="n"/>
+      <c r="AR14" s="16" t="n"/>
+      <c r="AS14" s="16" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="15" t="n"/>
@@ -2109,6 +2159,8 @@
       <c r="AO15" s="15" t="n"/>
       <c r="AP15" s="15" t="n"/>
       <c r="AQ15" s="16" t="n"/>
+      <c r="AR15" s="16" t="n"/>
+      <c r="AS15" s="16" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="n"/>
@@ -2162,6 +2214,8 @@
       <c r="AO16" s="15" t="n"/>
       <c r="AP16" s="15" t="n"/>
       <c r="AQ16" s="16" t="n"/>
+      <c r="AR16" s="16" t="n"/>
+      <c r="AS16" s="16" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="n"/>
@@ -2215,6 +2269,8 @@
       <c r="AO17" s="15" t="n"/>
       <c r="AP17" s="15" t="n"/>
       <c r="AQ17" s="16" t="n"/>
+      <c r="AR17" s="16" t="n"/>
+      <c r="AS17" s="16" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="n"/>
@@ -2268,6 +2324,8 @@
       <c r="AO18" s="15" t="n"/>
       <c r="AP18" s="15" t="n"/>
       <c r="AQ18" s="16" t="n"/>
+      <c r="AR18" s="16" t="n"/>
+      <c r="AS18" s="16" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="n"/>
@@ -2321,6 +2379,8 @@
       <c r="AO19" s="15" t="n"/>
       <c r="AP19" s="15" t="n"/>
       <c r="AQ19" s="16" t="n"/>
+      <c r="AR19" s="16" t="n"/>
+      <c r="AS19" s="16" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="15" t="n"/>
@@ -2374,6 +2434,8 @@
       <c r="AO20" s="15" t="n"/>
       <c r="AP20" s="15" t="n"/>
       <c r="AQ20" s="16" t="n"/>
+      <c r="AR20" s="16" t="n"/>
+      <c r="AS20" s="16" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="n"/>
@@ -2427,6 +2489,8 @@
       <c r="AO21" s="15" t="n"/>
       <c r="AP21" s="15" t="n"/>
       <c r="AQ21" s="16" t="n"/>
+      <c r="AR21" s="16" t="n"/>
+      <c r="AS21" s="16" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="n"/>
@@ -2480,6 +2544,8 @@
       <c r="AO22" s="15" t="n"/>
       <c r="AP22" s="15" t="n"/>
       <c r="AQ22" s="16" t="n"/>
+      <c r="AR22" s="16" t="n"/>
+      <c r="AS22" s="16" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="n"/>
@@ -2533,6 +2599,8 @@
       <c r="AO23" s="15" t="n"/>
       <c r="AP23" s="15" t="n"/>
       <c r="AQ23" s="16" t="n"/>
+      <c r="AR23" s="16" t="n"/>
+      <c r="AS23" s="16" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n"/>
@@ -2586,6 +2654,8 @@
       <c r="AO24" s="15" t="n"/>
       <c r="AP24" s="15" t="n"/>
       <c r="AQ24" s="16" t="n"/>
+      <c r="AR24" s="16" t="n"/>
+      <c r="AS24" s="16" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="15" t="n"/>
@@ -2639,6 +2709,8 @@
       <c r="AO25" s="15" t="n"/>
       <c r="AP25" s="15" t="n"/>
       <c r="AQ25" s="16" t="n"/>
+      <c r="AR25" s="16" t="n"/>
+      <c r="AS25" s="16" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="15" t="n"/>
@@ -2692,6 +2764,8 @@
       <c r="AO26" s="15" t="n"/>
       <c r="AP26" s="15" t="n"/>
       <c r="AQ26" s="16" t="n"/>
+      <c r="AR26" s="16" t="n"/>
+      <c r="AS26" s="16" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="15" t="n"/>
@@ -2745,6 +2819,8 @@
       <c r="AO27" s="15" t="n"/>
       <c r="AP27" s="15" t="n"/>
       <c r="AQ27" s="16" t="n"/>
+      <c r="AR27" s="16" t="n"/>
+      <c r="AS27" s="16" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="15" t="n"/>
@@ -2798,6 +2874,8 @@
       <c r="AO28" s="15" t="n"/>
       <c r="AP28" s="15" t="n"/>
       <c r="AQ28" s="16" t="n"/>
+      <c r="AR28" s="16" t="n"/>
+      <c r="AS28" s="16" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="15" t="n"/>
@@ -2851,6 +2929,8 @@
       <c r="AO29" s="15" t="n"/>
       <c r="AP29" s="15" t="n"/>
       <c r="AQ29" s="16" t="n"/>
+      <c r="AR29" s="16" t="n"/>
+      <c r="AS29" s="16" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="15" t="n"/>
@@ -2904,6 +2984,8 @@
       <c r="AO30" s="15" t="n"/>
       <c r="AP30" s="15" t="n"/>
       <c r="AQ30" s="16" t="n"/>
+      <c r="AR30" s="16" t="n"/>
+      <c r="AS30" s="16" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="15" t="n"/>
@@ -2957,6 +3039,8 @@
       <c r="AO31" s="15" t="n"/>
       <c r="AP31" s="15" t="n"/>
       <c r="AQ31" s="16" t="n"/>
+      <c r="AR31" s="16" t="n"/>
+      <c r="AS31" s="16" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="15" t="n"/>
@@ -3010,6 +3094,8 @@
       <c r="AO32" s="15" t="n"/>
       <c r="AP32" s="15" t="n"/>
       <c r="AQ32" s="16" t="n"/>
+      <c r="AR32" s="16" t="n"/>
+      <c r="AS32" s="16" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="15" t="n"/>
@@ -3063,6 +3149,8 @@
       <c r="AO33" s="15" t="n"/>
       <c r="AP33" s="15" t="n"/>
       <c r="AQ33" s="16" t="n"/>
+      <c r="AR33" s="16" t="n"/>
+      <c r="AS33" s="16" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="15" t="n"/>
@@ -3116,6 +3204,8 @@
       <c r="AO34" s="15" t="n"/>
       <c r="AP34" s="15" t="n"/>
       <c r="AQ34" s="16" t="n"/>
+      <c r="AR34" s="16" t="n"/>
+      <c r="AS34" s="16" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="15" t="n"/>
@@ -3169,6 +3259,8 @@
       <c r="AO35" s="15" t="n"/>
       <c r="AP35" s="15" t="n"/>
       <c r="AQ35" s="16" t="n"/>
+      <c r="AR35" s="16" t="n"/>
+      <c r="AS35" s="16" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="15" t="n"/>
@@ -3222,6 +3314,8 @@
       <c r="AO36" s="15" t="n"/>
       <c r="AP36" s="15" t="n"/>
       <c r="AQ36" s="16" t="n"/>
+      <c r="AR36" s="16" t="n"/>
+      <c r="AS36" s="16" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="15" t="n"/>
@@ -3275,6 +3369,8 @@
       <c r="AO37" s="15" t="n"/>
       <c r="AP37" s="15" t="n"/>
       <c r="AQ37" s="16" t="n"/>
+      <c r="AR37" s="16" t="n"/>
+      <c r="AS37" s="16" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="15" t="n"/>
@@ -3328,6 +3424,8 @@
       <c r="AO38" s="15" t="n"/>
       <c r="AP38" s="15" t="n"/>
       <c r="AQ38" s="16" t="n"/>
+      <c r="AR38" s="16" t="n"/>
+      <c r="AS38" s="16" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="15" t="n"/>
@@ -3381,6 +3479,8 @@
       <c r="AO39" s="15" t="n"/>
       <c r="AP39" s="15" t="n"/>
       <c r="AQ39" s="16" t="n"/>
+      <c r="AR39" s="16" t="n"/>
+      <c r="AS39" s="16" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="15" t="n"/>
@@ -3434,6 +3534,8 @@
       <c r="AO40" s="15" t="n"/>
       <c r="AP40" s="15" t="n"/>
       <c r="AQ40" s="16" t="n"/>
+      <c r="AR40" s="16" t="n"/>
+      <c r="AS40" s="16" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="15" t="n"/>
@@ -3487,6 +3589,8 @@
       <c r="AO41" s="15" t="n"/>
       <c r="AP41" s="15" t="n"/>
       <c r="AQ41" s="16" t="n"/>
+      <c r="AR41" s="16" t="n"/>
+      <c r="AS41" s="16" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="15" t="n"/>
@@ -3540,6 +3644,8 @@
       <c r="AO42" s="15" t="n"/>
       <c r="AP42" s="15" t="n"/>
       <c r="AQ42" s="16" t="n"/>
+      <c r="AR42" s="16" t="n"/>
+      <c r="AS42" s="16" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="15" t="n"/>
@@ -3593,6 +3699,8 @@
       <c r="AO43" s="15" t="n"/>
       <c r="AP43" s="15" t="n"/>
       <c r="AQ43" s="16" t="n"/>
+      <c r="AR43" s="16" t="n"/>
+      <c r="AS43" s="16" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="15" t="n"/>
@@ -3646,6 +3754,8 @@
       <c r="AO44" s="15" t="n"/>
       <c r="AP44" s="15" t="n"/>
       <c r="AQ44" s="16" t="n"/>
+      <c r="AR44" s="16" t="n"/>
+      <c r="AS44" s="16" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="15" t="n"/>
@@ -3699,6 +3809,8 @@
       <c r="AO45" s="15" t="n"/>
       <c r="AP45" s="15" t="n"/>
       <c r="AQ45" s="16" t="n"/>
+      <c r="AR45" s="16" t="n"/>
+      <c r="AS45" s="16" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="15" t="n"/>
@@ -3752,6 +3864,8 @@
       <c r="AO46" s="15" t="n"/>
       <c r="AP46" s="15" t="n"/>
       <c r="AQ46" s="16" t="n"/>
+      <c r="AR46" s="16" t="n"/>
+      <c r="AS46" s="16" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="15" t="n"/>
@@ -3805,6 +3919,8 @@
       <c r="AO47" s="15" t="n"/>
       <c r="AP47" s="15" t="n"/>
       <c r="AQ47" s="16" t="n"/>
+      <c r="AR47" s="16" t="n"/>
+      <c r="AS47" s="16" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="15" t="n"/>
@@ -3858,6 +3974,8 @@
       <c r="AO48" s="15" t="n"/>
       <c r="AP48" s="15" t="n"/>
       <c r="AQ48" s="16" t="n"/>
+      <c r="AR48" s="16" t="n"/>
+      <c r="AS48" s="16" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="15" t="n"/>
@@ -3911,6 +4029,8 @@
       <c r="AO49" s="15" t="n"/>
       <c r="AP49" s="15" t="n"/>
       <c r="AQ49" s="16" t="n"/>
+      <c r="AR49" s="16" t="n"/>
+      <c r="AS49" s="16" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="15" t="n"/>
@@ -3964,6 +4084,8 @@
       <c r="AO50" s="15" t="n"/>
       <c r="AP50" s="15" t="n"/>
       <c r="AQ50" s="16" t="n"/>
+      <c r="AR50" s="16" t="n"/>
+      <c r="AS50" s="16" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="15" t="n"/>
@@ -4017,6 +4139,8 @@
       <c r="AO51" s="15" t="n"/>
       <c r="AP51" s="15" t="n"/>
       <c r="AQ51" s="16" t="n"/>
+      <c r="AR51" s="16" t="n"/>
+      <c r="AS51" s="16" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="15" t="n"/>
@@ -4070,6 +4194,8 @@
       <c r="AO52" s="15" t="n"/>
       <c r="AP52" s="15" t="n"/>
       <c r="AQ52" s="16" t="n"/>
+      <c r="AR52" s="16" t="n"/>
+      <c r="AS52" s="16" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="15" t="n"/>
@@ -4123,6 +4249,8 @@
       <c r="AO53" s="15" t="n"/>
       <c r="AP53" s="15" t="n"/>
       <c r="AQ53" s="16" t="n"/>
+      <c r="AR53" s="16" t="n"/>
+      <c r="AS53" s="16" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="15" t="n"/>
@@ -4176,6 +4304,8 @@
       <c r="AO54" s="15" t="n"/>
       <c r="AP54" s="15" t="n"/>
       <c r="AQ54" s="16" t="n"/>
+      <c r="AR54" s="16" t="n"/>
+      <c r="AS54" s="16" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="15" t="n"/>
@@ -4229,6 +4359,8 @@
       <c r="AO55" s="15" t="n"/>
       <c r="AP55" s="15" t="n"/>
       <c r="AQ55" s="16" t="n"/>
+      <c r="AR55" s="16" t="n"/>
+      <c r="AS55" s="16" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="15" t="n"/>
@@ -4282,6 +4414,8 @@
       <c r="AO56" s="15" t="n"/>
       <c r="AP56" s="15" t="n"/>
       <c r="AQ56" s="16" t="n"/>
+      <c r="AR56" s="16" t="n"/>
+      <c r="AS56" s="16" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="15" t="n"/>
@@ -4335,6 +4469,8 @@
       <c r="AO57" s="15" t="n"/>
       <c r="AP57" s="15" t="n"/>
       <c r="AQ57" s="16" t="n"/>
+      <c r="AR57" s="16" t="n"/>
+      <c r="AS57" s="16" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="15" t="n"/>
@@ -4388,6 +4524,8 @@
       <c r="AO58" s="15" t="n"/>
       <c r="AP58" s="15" t="n"/>
       <c r="AQ58" s="16" t="n"/>
+      <c r="AR58" s="16" t="n"/>
+      <c r="AS58" s="16" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="15" t="n"/>
@@ -4441,6 +4579,8 @@
       <c r="AO59" s="15" t="n"/>
       <c r="AP59" s="15" t="n"/>
       <c r="AQ59" s="16" t="n"/>
+      <c r="AR59" s="16" t="n"/>
+      <c r="AS59" s="16" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="15" t="n"/>
@@ -4494,6 +4634,8 @@
       <c r="AO60" s="15" t="n"/>
       <c r="AP60" s="15" t="n"/>
       <c r="AQ60" s="16" t="n"/>
+      <c r="AR60" s="16" t="n"/>
+      <c r="AS60" s="16" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="15" t="n"/>
@@ -4547,6 +4689,8 @@
       <c r="AO61" s="15" t="n"/>
       <c r="AP61" s="15" t="n"/>
       <c r="AQ61" s="16" t="n"/>
+      <c r="AR61" s="16" t="n"/>
+      <c r="AS61" s="16" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="15" t="n"/>
@@ -4600,6 +4744,8 @@
       <c r="AO62" s="15" t="n"/>
       <c r="AP62" s="15" t="n"/>
       <c r="AQ62" s="16" t="n"/>
+      <c r="AR62" s="16" t="n"/>
+      <c r="AS62" s="16" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="15" t="n"/>
@@ -4653,6 +4799,8 @@
       <c r="AO63" s="15" t="n"/>
       <c r="AP63" s="15" t="n"/>
       <c r="AQ63" s="16" t="n"/>
+      <c r="AR63" s="16" t="n"/>
+      <c r="AS63" s="16" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="15" t="n"/>
@@ -4706,6 +4854,8 @@
       <c r="AO64" s="15" t="n"/>
       <c r="AP64" s="15" t="n"/>
       <c r="AQ64" s="16" t="n"/>
+      <c r="AR64" s="16" t="n"/>
+      <c r="AS64" s="16" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="15" t="n"/>
@@ -4759,6 +4909,8 @@
       <c r="AO65" s="15" t="n"/>
       <c r="AP65" s="15" t="n"/>
       <c r="AQ65" s="16" t="n"/>
+      <c r="AR65" s="16" t="n"/>
+      <c r="AS65" s="16" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="15" t="n"/>
@@ -4812,6 +4964,8 @@
       <c r="AO66" s="15" t="n"/>
       <c r="AP66" s="15" t="n"/>
       <c r="AQ66" s="16" t="n"/>
+      <c r="AR66" s="16" t="n"/>
+      <c r="AS66" s="16" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="15" t="n"/>
@@ -4865,6 +5019,8 @@
       <c r="AO67" s="15" t="n"/>
       <c r="AP67" s="15" t="n"/>
       <c r="AQ67" s="16" t="n"/>
+      <c r="AR67" s="16" t="n"/>
+      <c r="AS67" s="16" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="15" t="n"/>
@@ -4918,6 +5074,8 @@
       <c r="AO68" s="15" t="n"/>
       <c r="AP68" s="15" t="n"/>
       <c r="AQ68" s="16" t="n"/>
+      <c r="AR68" s="16" t="n"/>
+      <c r="AS68" s="16" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="15" t="n"/>
@@ -4971,6 +5129,8 @@
       <c r="AO69" s="15" t="n"/>
       <c r="AP69" s="15" t="n"/>
       <c r="AQ69" s="16" t="n"/>
+      <c r="AR69" s="16" t="n"/>
+      <c r="AS69" s="16" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="15" t="n"/>
@@ -5024,6 +5184,8 @@
       <c r="AO70" s="15" t="n"/>
       <c r="AP70" s="15" t="n"/>
       <c r="AQ70" s="16" t="n"/>
+      <c r="AR70" s="16" t="n"/>
+      <c r="AS70" s="16" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="15" t="n"/>
@@ -5077,6 +5239,8 @@
       <c r="AO71" s="15" t="n"/>
       <c r="AP71" s="15" t="n"/>
       <c r="AQ71" s="16" t="n"/>
+      <c r="AR71" s="16" t="n"/>
+      <c r="AS71" s="16" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="15" t="n"/>
@@ -5130,6 +5294,8 @@
       <c r="AO72" s="15" t="n"/>
       <c r="AP72" s="15" t="n"/>
       <c r="AQ72" s="16" t="n"/>
+      <c r="AR72" s="16" t="n"/>
+      <c r="AS72" s="16" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="15" t="n"/>
@@ -5183,6 +5349,8 @@
       <c r="AO73" s="15" t="n"/>
       <c r="AP73" s="15" t="n"/>
       <c r="AQ73" s="16" t="n"/>
+      <c r="AR73" s="16" t="n"/>
+      <c r="AS73" s="16" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="15" t="n"/>
@@ -5236,6 +5404,8 @@
       <c r="AO74" s="15" t="n"/>
       <c r="AP74" s="15" t="n"/>
       <c r="AQ74" s="16" t="n"/>
+      <c r="AR74" s="16" t="n"/>
+      <c r="AS74" s="16" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="15" t="n"/>
@@ -5289,6 +5459,8 @@
       <c r="AO75" s="15" t="n"/>
       <c r="AP75" s="15" t="n"/>
       <c r="AQ75" s="16" t="n"/>
+      <c r="AR75" s="16" t="n"/>
+      <c r="AS75" s="16" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="15" t="n"/>
@@ -5342,6 +5514,8 @@
       <c r="AO76" s="15" t="n"/>
       <c r="AP76" s="15" t="n"/>
       <c r="AQ76" s="16" t="n"/>
+      <c r="AR76" s="16" t="n"/>
+      <c r="AS76" s="16" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="15" t="n"/>
@@ -5395,6 +5569,8 @@
       <c r="AO77" s="15" t="n"/>
       <c r="AP77" s="15" t="n"/>
       <c r="AQ77" s="16" t="n"/>
+      <c r="AR77" s="16" t="n"/>
+      <c r="AS77" s="16" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="15" t="n"/>
@@ -5448,6 +5624,8 @@
       <c r="AO78" s="15" t="n"/>
       <c r="AP78" s="15" t="n"/>
       <c r="AQ78" s="16" t="n"/>
+      <c r="AR78" s="16" t="n"/>
+      <c r="AS78" s="16" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="15" t="n"/>
@@ -5501,6 +5679,8 @@
       <c r="AO79" s="15" t="n"/>
       <c r="AP79" s="15" t="n"/>
       <c r="AQ79" s="16" t="n"/>
+      <c r="AR79" s="16" t="n"/>
+      <c r="AS79" s="16" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="15" t="n"/>
@@ -5554,6 +5734,8 @@
       <c r="AO80" s="15" t="n"/>
       <c r="AP80" s="15" t="n"/>
       <c r="AQ80" s="16" t="n"/>
+      <c r="AR80" s="16" t="n"/>
+      <c r="AS80" s="16" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="15" t="n"/>
@@ -5607,6 +5789,8 @@
       <c r="AO81" s="15" t="n"/>
       <c r="AP81" s="15" t="n"/>
       <c r="AQ81" s="16" t="n"/>
+      <c r="AR81" s="16" t="n"/>
+      <c r="AS81" s="16" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="15" t="n"/>
@@ -5660,6 +5844,8 @@
       <c r="AO82" s="15" t="n"/>
       <c r="AP82" s="15" t="n"/>
       <c r="AQ82" s="16" t="n"/>
+      <c r="AR82" s="16" t="n"/>
+      <c r="AS82" s="16" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="15" t="n"/>
@@ -5713,6 +5899,8 @@
       <c r="AO83" s="15" t="n"/>
       <c r="AP83" s="15" t="n"/>
       <c r="AQ83" s="16" t="n"/>
+      <c r="AR83" s="16" t="n"/>
+      <c r="AS83" s="16" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="15" t="n"/>
@@ -5766,6 +5954,8 @@
       <c r="AO84" s="15" t="n"/>
       <c r="AP84" s="15" t="n"/>
       <c r="AQ84" s="16" t="n"/>
+      <c r="AR84" s="16" t="n"/>
+      <c r="AS84" s="16" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="15" t="n"/>
@@ -5819,6 +6009,8 @@
       <c r="AO85" s="15" t="n"/>
       <c r="AP85" s="15" t="n"/>
       <c r="AQ85" s="16" t="n"/>
+      <c r="AR85" s="16" t="n"/>
+      <c r="AS85" s="16" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="15" t="n"/>
@@ -5872,6 +6064,8 @@
       <c r="AO86" s="15" t="n"/>
       <c r="AP86" s="15" t="n"/>
       <c r="AQ86" s="16" t="n"/>
+      <c r="AR86" s="16" t="n"/>
+      <c r="AS86" s="16" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="15" t="n"/>
@@ -5925,6 +6119,8 @@
       <c r="AO87" s="15" t="n"/>
       <c r="AP87" s="15" t="n"/>
       <c r="AQ87" s="16" t="n"/>
+      <c r="AR87" s="16" t="n"/>
+      <c r="AS87" s="16" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="15" t="n"/>
@@ -5978,6 +6174,8 @@
       <c r="AO88" s="15" t="n"/>
       <c r="AP88" s="15" t="n"/>
       <c r="AQ88" s="16" t="n"/>
+      <c r="AR88" s="16" t="n"/>
+      <c r="AS88" s="16" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="15" t="n"/>
@@ -6031,6 +6229,8 @@
       <c r="AO89" s="15" t="n"/>
       <c r="AP89" s="15" t="n"/>
       <c r="AQ89" s="16" t="n"/>
+      <c r="AR89" s="16" t="n"/>
+      <c r="AS89" s="16" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="15" t="n"/>
@@ -6084,6 +6284,8 @@
       <c r="AO90" s="15" t="n"/>
       <c r="AP90" s="15" t="n"/>
       <c r="AQ90" s="16" t="n"/>
+      <c r="AR90" s="16" t="n"/>
+      <c r="AS90" s="16" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="15" t="n"/>
@@ -6137,6 +6339,8 @@
       <c r="AO91" s="15" t="n"/>
       <c r="AP91" s="15" t="n"/>
       <c r="AQ91" s="16" t="n"/>
+      <c r="AR91" s="16" t="n"/>
+      <c r="AS91" s="16" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="15" t="n"/>
@@ -6190,6 +6394,8 @@
       <c r="AO92" s="15" t="n"/>
       <c r="AP92" s="15" t="n"/>
       <c r="AQ92" s="16" t="n"/>
+      <c r="AR92" s="16" t="n"/>
+      <c r="AS92" s="16" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="15" t="n"/>
@@ -6243,6 +6449,8 @@
       <c r="AO93" s="15" t="n"/>
       <c r="AP93" s="15" t="n"/>
       <c r="AQ93" s="16" t="n"/>
+      <c r="AR93" s="16" t="n"/>
+      <c r="AS93" s="16" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="15" t="n"/>
@@ -6296,6 +6504,8 @@
       <c r="AO94" s="15" t="n"/>
       <c r="AP94" s="15" t="n"/>
       <c r="AQ94" s="16" t="n"/>
+      <c r="AR94" s="16" t="n"/>
+      <c r="AS94" s="16" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="15" t="n"/>
@@ -6349,6 +6559,8 @@
       <c r="AO95" s="15" t="n"/>
       <c r="AP95" s="15" t="n"/>
       <c r="AQ95" s="16" t="n"/>
+      <c r="AR95" s="16" t="n"/>
+      <c r="AS95" s="16" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="15" t="n"/>
@@ -6402,6 +6614,8 @@
       <c r="AO96" s="15" t="n"/>
       <c r="AP96" s="15" t="n"/>
       <c r="AQ96" s="16" t="n"/>
+      <c r="AR96" s="16" t="n"/>
+      <c r="AS96" s="16" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="15" t="n"/>
@@ -6455,6 +6669,8 @@
       <c r="AO97" s="15" t="n"/>
       <c r="AP97" s="15" t="n"/>
       <c r="AQ97" s="16" t="n"/>
+      <c r="AR97" s="16" t="n"/>
+      <c r="AS97" s="16" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="15" t="n"/>
@@ -6508,6 +6724,8 @@
       <c r="AO98" s="15" t="n"/>
       <c r="AP98" s="15" t="n"/>
       <c r="AQ98" s="16" t="n"/>
+      <c r="AR98" s="16" t="n"/>
+      <c r="AS98" s="16" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="15" t="n"/>
@@ -6561,6 +6779,8 @@
       <c r="AO99" s="15" t="n"/>
       <c r="AP99" s="15" t="n"/>
       <c r="AQ99" s="16" t="n"/>
+      <c r="AR99" s="16" t="n"/>
+      <c r="AS99" s="16" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="15" t="n"/>
@@ -6614,6 +6834,8 @@
       <c r="AO100" s="15" t="n"/>
       <c r="AP100" s="15" t="n"/>
       <c r="AQ100" s="16" t="n"/>
+      <c r="AR100" s="16" t="n"/>
+      <c r="AS100" s="16" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="15" t="n"/>
@@ -6667,6 +6889,8 @@
       <c r="AO101" s="15" t="n"/>
       <c r="AP101" s="15" t="n"/>
       <c r="AQ101" s="16" t="n"/>
+      <c r="AR101" s="16" t="n"/>
+      <c r="AS101" s="16" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="15" t="n"/>
@@ -6720,6 +6944,8 @@
       <c r="AO102" s="15" t="n"/>
       <c r="AP102" s="15" t="n"/>
       <c r="AQ102" s="16" t="n"/>
+      <c r="AR102" s="16" t="n"/>
+      <c r="AS102" s="16" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="15" t="n"/>
@@ -6773,6 +6999,8 @@
       <c r="AO103" s="15" t="n"/>
       <c r="AP103" s="15" t="n"/>
       <c r="AQ103" s="16" t="n"/>
+      <c r="AR103" s="16" t="n"/>
+      <c r="AS103" s="16" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="15" t="n"/>
@@ -6826,6 +7054,8 @@
       <c r="AO104" s="15" t="n"/>
       <c r="AP104" s="15" t="n"/>
       <c r="AQ104" s="16" t="n"/>
+      <c r="AR104" s="16" t="n"/>
+      <c r="AS104" s="16" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="15" t="n"/>
@@ -6879,6 +7109,8 @@
       <c r="AO105" s="15" t="n"/>
       <c r="AP105" s="15" t="n"/>
       <c r="AQ105" s="16" t="n"/>
+      <c r="AR105" s="16" t="n"/>
+      <c r="AS105" s="16" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="15" t="n"/>
@@ -6932,6 +7164,8 @@
       <c r="AO106" s="15" t="n"/>
       <c r="AP106" s="15" t="n"/>
       <c r="AQ106" s="16" t="n"/>
+      <c r="AR106" s="16" t="n"/>
+      <c r="AS106" s="16" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="15" t="n"/>
@@ -6985,6 +7219,8 @@
       <c r="AO107" s="15" t="n"/>
       <c r="AP107" s="15" t="n"/>
       <c r="AQ107" s="16" t="n"/>
+      <c r="AR107" s="16" t="n"/>
+      <c r="AS107" s="16" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="15" t="n"/>
@@ -7038,6 +7274,8 @@
       <c r="AO108" s="15" t="n"/>
       <c r="AP108" s="15" t="n"/>
       <c r="AQ108" s="16" t="n"/>
+      <c r="AR108" s="16" t="n"/>
+      <c r="AS108" s="16" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="15" t="n"/>
@@ -7091,6 +7329,8 @@
       <c r="AO109" s="15" t="n"/>
       <c r="AP109" s="15" t="n"/>
       <c r="AQ109" s="16" t="n"/>
+      <c r="AR109" s="16" t="n"/>
+      <c r="AS109" s="16" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="15" t="n"/>
@@ -7144,6 +7384,8 @@
       <c r="AO110" s="15" t="n"/>
       <c r="AP110" s="15" t="n"/>
       <c r="AQ110" s="16" t="n"/>
+      <c r="AR110" s="16" t="n"/>
+      <c r="AS110" s="16" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="15" t="n"/>
@@ -7197,6 +7439,8 @@
       <c r="AO111" s="15" t="n"/>
       <c r="AP111" s="15" t="n"/>
       <c r="AQ111" s="16" t="n"/>
+      <c r="AR111" s="16" t="n"/>
+      <c r="AS111" s="16" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="15" t="n"/>
@@ -7250,6 +7494,8 @@
       <c r="AO112" s="15" t="n"/>
       <c r="AP112" s="15" t="n"/>
       <c r="AQ112" s="16" t="n"/>
+      <c r="AR112" s="16" t="n"/>
+      <c r="AS112" s="16" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="15" t="n"/>
@@ -7303,6 +7549,8 @@
       <c r="AO113" s="15" t="n"/>
       <c r="AP113" s="15" t="n"/>
       <c r="AQ113" s="16" t="n"/>
+      <c r="AR113" s="16" t="n"/>
+      <c r="AS113" s="16" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="15" t="n"/>
@@ -7356,6 +7604,8 @@
       <c r="AO114" s="15" t="n"/>
       <c r="AP114" s="15" t="n"/>
       <c r="AQ114" s="16" t="n"/>
+      <c r="AR114" s="16" t="n"/>
+      <c r="AS114" s="16" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="15" t="n"/>
@@ -7409,6 +7659,8 @@
       <c r="AO115" s="15" t="n"/>
       <c r="AP115" s="15" t="n"/>
       <c r="AQ115" s="16" t="n"/>
+      <c r="AR115" s="16" t="n"/>
+      <c r="AS115" s="16" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="15" t="n"/>
@@ -7462,6 +7714,8 @@
       <c r="AO116" s="15" t="n"/>
       <c r="AP116" s="15" t="n"/>
       <c r="AQ116" s="16" t="n"/>
+      <c r="AR116" s="16" t="n"/>
+      <c r="AS116" s="16" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="15" t="n"/>
@@ -7515,6 +7769,8 @@
       <c r="AO117" s="15" t="n"/>
       <c r="AP117" s="15" t="n"/>
       <c r="AQ117" s="16" t="n"/>
+      <c r="AR117" s="16" t="n"/>
+      <c r="AS117" s="16" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="15" t="n"/>
@@ -7568,6 +7824,8 @@
       <c r="AO118" s="15" t="n"/>
       <c r="AP118" s="15" t="n"/>
       <c r="AQ118" s="16" t="n"/>
+      <c r="AR118" s="16" t="n"/>
+      <c r="AS118" s="16" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="15" t="n"/>
@@ -7621,6 +7879,8 @@
       <c r="AO119" s="15" t="n"/>
       <c r="AP119" s="15" t="n"/>
       <c r="AQ119" s="16" t="n"/>
+      <c r="AR119" s="16" t="n"/>
+      <c r="AS119" s="16" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="15" t="n"/>
@@ -7674,6 +7934,8 @@
       <c r="AO120" s="15" t="n"/>
       <c r="AP120" s="15" t="n"/>
       <c r="AQ120" s="16" t="n"/>
+      <c r="AR120" s="16" t="n"/>
+      <c r="AS120" s="16" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="15" t="n"/>
@@ -7727,6 +7989,8 @@
       <c r="AO121" s="15" t="n"/>
       <c r="AP121" s="15" t="n"/>
       <c r="AQ121" s="16" t="n"/>
+      <c r="AR121" s="16" t="n"/>
+      <c r="AS121" s="16" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="15" t="n"/>
@@ -7780,6 +8044,8 @@
       <c r="AO122" s="15" t="n"/>
       <c r="AP122" s="15" t="n"/>
       <c r="AQ122" s="16" t="n"/>
+      <c r="AR122" s="16" t="n"/>
+      <c r="AS122" s="16" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="15" t="n"/>
@@ -7833,6 +8099,8 @@
       <c r="AO123" s="15" t="n"/>
       <c r="AP123" s="15" t="n"/>
       <c r="AQ123" s="16" t="n"/>
+      <c r="AR123" s="16" t="n"/>
+      <c r="AS123" s="16" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="15" t="n"/>
@@ -7886,6 +8154,8 @@
       <c r="AO124" s="15" t="n"/>
       <c r="AP124" s="15" t="n"/>
       <c r="AQ124" s="16" t="n"/>
+      <c r="AR124" s="16" t="n"/>
+      <c r="AS124" s="16" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="15" t="n"/>
@@ -7939,6 +8209,8 @@
       <c r="AO125" s="15" t="n"/>
       <c r="AP125" s="15" t="n"/>
       <c r="AQ125" s="16" t="n"/>
+      <c r="AR125" s="16" t="n"/>
+      <c r="AS125" s="16" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="15" t="n"/>
@@ -7992,6 +8264,8 @@
       <c r="AO126" s="15" t="n"/>
       <c r="AP126" s="15" t="n"/>
       <c r="AQ126" s="16" t="n"/>
+      <c r="AR126" s="16" t="n"/>
+      <c r="AS126" s="16" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="15" t="n"/>
@@ -8045,6 +8319,8 @@
       <c r="AO127" s="15" t="n"/>
       <c r="AP127" s="15" t="n"/>
       <c r="AQ127" s="16" t="n"/>
+      <c r="AR127" s="16" t="n"/>
+      <c r="AS127" s="16" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="15" t="n"/>
@@ -8098,6 +8374,8 @@
       <c r="AO128" s="15" t="n"/>
       <c r="AP128" s="15" t="n"/>
       <c r="AQ128" s="16" t="n"/>
+      <c r="AR128" s="16" t="n"/>
+      <c r="AS128" s="16" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="15" t="n"/>
@@ -8151,6 +8429,8 @@
       <c r="AO129" s="15" t="n"/>
       <c r="AP129" s="15" t="n"/>
       <c r="AQ129" s="16" t="n"/>
+      <c r="AR129" s="16" t="n"/>
+      <c r="AS129" s="16" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="15" t="n"/>
@@ -8204,6 +8484,8 @@
       <c r="AO130" s="15" t="n"/>
       <c r="AP130" s="15" t="n"/>
       <c r="AQ130" s="16" t="n"/>
+      <c r="AR130" s="16" t="n"/>
+      <c r="AS130" s="16" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="15" t="n"/>
@@ -8257,6 +8539,8 @@
       <c r="AO131" s="15" t="n"/>
       <c r="AP131" s="15" t="n"/>
       <c r="AQ131" s="16" t="n"/>
+      <c r="AR131" s="16" t="n"/>
+      <c r="AS131" s="16" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="15" t="n"/>
@@ -8310,6 +8594,8 @@
       <c r="AO132" s="15" t="n"/>
       <c r="AP132" s="15" t="n"/>
       <c r="AQ132" s="16" t="n"/>
+      <c r="AR132" s="16" t="n"/>
+      <c r="AS132" s="16" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="15" t="n"/>
@@ -8363,6 +8649,8 @@
       <c r="AO133" s="15" t="n"/>
       <c r="AP133" s="15" t="n"/>
       <c r="AQ133" s="16" t="n"/>
+      <c r="AR133" s="16" t="n"/>
+      <c r="AS133" s="16" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="15" t="n"/>
@@ -8416,6 +8704,8 @@
       <c r="AO134" s="15" t="n"/>
       <c r="AP134" s="15" t="n"/>
       <c r="AQ134" s="16" t="n"/>
+      <c r="AR134" s="16" t="n"/>
+      <c r="AS134" s="16" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="15" t="n"/>
@@ -8469,6 +8759,8 @@
       <c r="AO135" s="15" t="n"/>
       <c r="AP135" s="15" t="n"/>
       <c r="AQ135" s="16" t="n"/>
+      <c r="AR135" s="16" t="n"/>
+      <c r="AS135" s="16" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="15" t="n"/>
@@ -8522,6 +8814,8 @@
       <c r="AO136" s="15" t="n"/>
       <c r="AP136" s="15" t="n"/>
       <c r="AQ136" s="16" t="n"/>
+      <c r="AR136" s="16" t="n"/>
+      <c r="AS136" s="16" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="15" t="n"/>
@@ -8575,6 +8869,8 @@
       <c r="AO137" s="15" t="n"/>
       <c r="AP137" s="15" t="n"/>
       <c r="AQ137" s="16" t="n"/>
+      <c r="AR137" s="16" t="n"/>
+      <c r="AS137" s="16" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="15" t="n"/>
@@ -8628,6 +8924,8 @@
       <c r="AO138" s="15" t="n"/>
       <c r="AP138" s="15" t="n"/>
       <c r="AQ138" s="16" t="n"/>
+      <c r="AR138" s="16" t="n"/>
+      <c r="AS138" s="16" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="15" t="n"/>
@@ -8681,6 +8979,8 @@
       <c r="AO139" s="15" t="n"/>
       <c r="AP139" s="15" t="n"/>
       <c r="AQ139" s="16" t="n"/>
+      <c r="AR139" s="16" t="n"/>
+      <c r="AS139" s="16" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="15" t="n"/>
@@ -8734,6 +9034,8 @@
       <c r="AO140" s="15" t="n"/>
       <c r="AP140" s="15" t="n"/>
       <c r="AQ140" s="16" t="n"/>
+      <c r="AR140" s="16" t="n"/>
+      <c r="AS140" s="16" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="15" t="n"/>
@@ -8787,6 +9089,8 @@
       <c r="AO141" s="15" t="n"/>
       <c r="AP141" s="15" t="n"/>
       <c r="AQ141" s="16" t="n"/>
+      <c r="AR141" s="16" t="n"/>
+      <c r="AS141" s="16" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="15" t="n"/>
@@ -8840,6 +9144,8 @@
       <c r="AO142" s="15" t="n"/>
       <c r="AP142" s="15" t="n"/>
       <c r="AQ142" s="16" t="n"/>
+      <c r="AR142" s="16" t="n"/>
+      <c r="AS142" s="16" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="15" t="n"/>
@@ -8893,6 +9199,8 @@
       <c r="AO143" s="15" t="n"/>
       <c r="AP143" s="15" t="n"/>
       <c r="AQ143" s="16" t="n"/>
+      <c r="AR143" s="16" t="n"/>
+      <c r="AS143" s="16" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="15" t="n"/>
@@ -8946,6 +9254,8 @@
       <c r="AO144" s="15" t="n"/>
       <c r="AP144" s="15" t="n"/>
       <c r="AQ144" s="16" t="n"/>
+      <c r="AR144" s="16" t="n"/>
+      <c r="AS144" s="16" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="15" t="n"/>
@@ -8999,6 +9309,8 @@
       <c r="AO145" s="15" t="n"/>
       <c r="AP145" s="15" t="n"/>
       <c r="AQ145" s="16" t="n"/>
+      <c r="AR145" s="16" t="n"/>
+      <c r="AS145" s="16" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="15" t="n"/>
@@ -9052,6 +9364,8 @@
       <c r="AO146" s="15" t="n"/>
       <c r="AP146" s="15" t="n"/>
       <c r="AQ146" s="16" t="n"/>
+      <c r="AR146" s="16" t="n"/>
+      <c r="AS146" s="16" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="15" t="n"/>
@@ -9105,6 +9419,8 @@
       <c r="AO147" s="15" t="n"/>
       <c r="AP147" s="15" t="n"/>
       <c r="AQ147" s="16" t="n"/>
+      <c r="AR147" s="16" t="n"/>
+      <c r="AS147" s="16" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="15" t="n"/>
@@ -9158,6 +9474,8 @@
       <c r="AO148" s="15" t="n"/>
       <c r="AP148" s="15" t="n"/>
       <c r="AQ148" s="16" t="n"/>
+      <c r="AR148" s="16" t="n"/>
+      <c r="AS148" s="16" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="15" t="n"/>
@@ -9211,6 +9529,8 @@
       <c r="AO149" s="15" t="n"/>
       <c r="AP149" s="15" t="n"/>
       <c r="AQ149" s="16" t="n"/>
+      <c r="AR149" s="16" t="n"/>
+      <c r="AS149" s="16" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="15" t="n"/>
@@ -9264,6 +9584,8 @@
       <c r="AO150" s="15" t="n"/>
       <c r="AP150" s="15" t="n"/>
       <c r="AQ150" s="16" t="n"/>
+      <c r="AR150" s="16" t="n"/>
+      <c r="AS150" s="16" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="15" t="n"/>
@@ -9317,6 +9639,8 @@
       <c r="AO151" s="15" t="n"/>
       <c r="AP151" s="15" t="n"/>
       <c r="AQ151" s="16" t="n"/>
+      <c r="AR151" s="16" t="n"/>
+      <c r="AS151" s="16" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="15" t="n"/>
@@ -9370,6 +9694,8 @@
       <c r="AO152" s="15" t="n"/>
       <c r="AP152" s="15" t="n"/>
       <c r="AQ152" s="16" t="n"/>
+      <c r="AR152" s="16" t="n"/>
+      <c r="AS152" s="16" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="15" t="n"/>
@@ -9423,6 +9749,8 @@
       <c r="AO153" s="15" t="n"/>
       <c r="AP153" s="15" t="n"/>
       <c r="AQ153" s="16" t="n"/>
+      <c r="AR153" s="16" t="n"/>
+      <c r="AS153" s="16" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="15" t="n"/>
@@ -9476,6 +9804,8 @@
       <c r="AO154" s="15" t="n"/>
       <c r="AP154" s="15" t="n"/>
       <c r="AQ154" s="16" t="n"/>
+      <c r="AR154" s="16" t="n"/>
+      <c r="AS154" s="16" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="15" t="n"/>
@@ -9529,6 +9859,8 @@
       <c r="AO155" s="15" t="n"/>
       <c r="AP155" s="15" t="n"/>
       <c r="AQ155" s="16" t="n"/>
+      <c r="AR155" s="16" t="n"/>
+      <c r="AS155" s="16" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="15" t="n"/>
@@ -9582,6 +9914,8 @@
       <c r="AO156" s="15" t="n"/>
       <c r="AP156" s="15" t="n"/>
       <c r="AQ156" s="16" t="n"/>
+      <c r="AR156" s="16" t="n"/>
+      <c r="AS156" s="16" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="15" t="n"/>
@@ -9635,6 +9969,8 @@
       <c r="AO157" s="15" t="n"/>
       <c r="AP157" s="15" t="n"/>
       <c r="AQ157" s="16" t="n"/>
+      <c r="AR157" s="16" t="n"/>
+      <c r="AS157" s="16" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="15" t="n"/>
@@ -9688,6 +10024,8 @@
       <c r="AO158" s="15" t="n"/>
       <c r="AP158" s="15" t="n"/>
       <c r="AQ158" s="16" t="n"/>
+      <c r="AR158" s="16" t="n"/>
+      <c r="AS158" s="16" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="15" t="n"/>
@@ -9741,6 +10079,8 @@
       <c r="AO159" s="15" t="n"/>
       <c r="AP159" s="15" t="n"/>
       <c r="AQ159" s="16" t="n"/>
+      <c r="AR159" s="16" t="n"/>
+      <c r="AS159" s="16" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="15" t="n"/>
@@ -9794,6 +10134,8 @@
       <c r="AO160" s="15" t="n"/>
       <c r="AP160" s="15" t="n"/>
       <c r="AQ160" s="16" t="n"/>
+      <c r="AR160" s="16" t="n"/>
+      <c r="AS160" s="16" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="15" t="n"/>
@@ -9847,6 +10189,8 @@
       <c r="AO161" s="15" t="n"/>
       <c r="AP161" s="15" t="n"/>
       <c r="AQ161" s="16" t="n"/>
+      <c r="AR161" s="16" t="n"/>
+      <c r="AS161" s="16" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="15" t="n"/>
@@ -9900,6 +10244,8 @@
       <c r="AO162" s="15" t="n"/>
       <c r="AP162" s="15" t="n"/>
       <c r="AQ162" s="16" t="n"/>
+      <c r="AR162" s="16" t="n"/>
+      <c r="AS162" s="16" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="15" t="n"/>
@@ -9953,6 +10299,8 @@
       <c r="AO163" s="15" t="n"/>
       <c r="AP163" s="15" t="n"/>
       <c r="AQ163" s="16" t="n"/>
+      <c r="AR163" s="16" t="n"/>
+      <c r="AS163" s="16" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="15" t="n"/>
@@ -10006,6 +10354,8 @@
       <c r="AO164" s="15" t="n"/>
       <c r="AP164" s="15" t="n"/>
       <c r="AQ164" s="16" t="n"/>
+      <c r="AR164" s="16" t="n"/>
+      <c r="AS164" s="16" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="15" t="n"/>
@@ -10059,6 +10409,8 @@
       <c r="AO165" s="15" t="n"/>
       <c r="AP165" s="15" t="n"/>
       <c r="AQ165" s="16" t="n"/>
+      <c r="AR165" s="16" t="n"/>
+      <c r="AS165" s="16" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="15" t="n"/>
@@ -10112,6 +10464,8 @@
       <c r="AO166" s="15" t="n"/>
       <c r="AP166" s="15" t="n"/>
       <c r="AQ166" s="16" t="n"/>
+      <c r="AR166" s="16" t="n"/>
+      <c r="AS166" s="16" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="15" t="n"/>
@@ -10165,6 +10519,8 @@
       <c r="AO167" s="15" t="n"/>
       <c r="AP167" s="15" t="n"/>
       <c r="AQ167" s="16" t="n"/>
+      <c r="AR167" s="16" t="n"/>
+      <c r="AS167" s="16" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="15" t="n"/>
@@ -10218,6 +10574,8 @@
       <c r="AO168" s="15" t="n"/>
       <c r="AP168" s="15" t="n"/>
       <c r="AQ168" s="16" t="n"/>
+      <c r="AR168" s="16" t="n"/>
+      <c r="AS168" s="16" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="15" t="n"/>
@@ -10271,6 +10629,8 @@
       <c r="AO169" s="15" t="n"/>
       <c r="AP169" s="15" t="n"/>
       <c r="AQ169" s="16" t="n"/>
+      <c r="AR169" s="16" t="n"/>
+      <c r="AS169" s="16" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="15" t="n"/>
@@ -10324,6 +10684,8 @@
       <c r="AO170" s="15" t="n"/>
       <c r="AP170" s="15" t="n"/>
       <c r="AQ170" s="16" t="n"/>
+      <c r="AR170" s="16" t="n"/>
+      <c r="AS170" s="16" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="15" t="n"/>
@@ -10377,6 +10739,8 @@
       <c r="AO171" s="15" t="n"/>
       <c r="AP171" s="15" t="n"/>
       <c r="AQ171" s="16" t="n"/>
+      <c r="AR171" s="16" t="n"/>
+      <c r="AS171" s="16" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="15" t="n"/>
@@ -10430,6 +10794,8 @@
       <c r="AO172" s="15" t="n"/>
       <c r="AP172" s="15" t="n"/>
       <c r="AQ172" s="16" t="n"/>
+      <c r="AR172" s="16" t="n"/>
+      <c r="AS172" s="16" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="15" t="n"/>
@@ -10483,6 +10849,8 @@
       <c r="AO173" s="15" t="n"/>
       <c r="AP173" s="15" t="n"/>
       <c r="AQ173" s="16" t="n"/>
+      <c r="AR173" s="16" t="n"/>
+      <c r="AS173" s="16" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="15" t="n"/>
@@ -10536,6 +10904,8 @@
       <c r="AO174" s="15" t="n"/>
       <c r="AP174" s="15" t="n"/>
       <c r="AQ174" s="16" t="n"/>
+      <c r="AR174" s="16" t="n"/>
+      <c r="AS174" s="16" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="15" t="n"/>
@@ -10589,6 +10959,8 @@
       <c r="AO175" s="15" t="n"/>
       <c r="AP175" s="15" t="n"/>
       <c r="AQ175" s="16" t="n"/>
+      <c r="AR175" s="16" t="n"/>
+      <c r="AS175" s="16" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="15" t="n"/>
@@ -10642,6 +11014,8 @@
       <c r="AO176" s="15" t="n"/>
       <c r="AP176" s="15" t="n"/>
       <c r="AQ176" s="16" t="n"/>
+      <c r="AR176" s="16" t="n"/>
+      <c r="AS176" s="16" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="15" t="n"/>
@@ -10695,6 +11069,8 @@
       <c r="AO177" s="15" t="n"/>
       <c r="AP177" s="15" t="n"/>
       <c r="AQ177" s="16" t="n"/>
+      <c r="AR177" s="16" t="n"/>
+      <c r="AS177" s="16" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="15" t="n"/>
@@ -10748,6 +11124,8 @@
       <c r="AO178" s="15" t="n"/>
       <c r="AP178" s="15" t="n"/>
       <c r="AQ178" s="16" t="n"/>
+      <c r="AR178" s="16" t="n"/>
+      <c r="AS178" s="16" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="15" t="n"/>
@@ -10801,6 +11179,8 @@
       <c r="AO179" s="15" t="n"/>
       <c r="AP179" s="15" t="n"/>
       <c r="AQ179" s="16" t="n"/>
+      <c r="AR179" s="16" t="n"/>
+      <c r="AS179" s="16" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="15" t="n"/>
@@ -10854,6 +11234,8 @@
       <c r="AO180" s="15" t="n"/>
       <c r="AP180" s="15" t="n"/>
       <c r="AQ180" s="16" t="n"/>
+      <c r="AR180" s="16" t="n"/>
+      <c r="AS180" s="16" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="15" t="n"/>
@@ -10907,6 +11289,8 @@
       <c r="AO181" s="15" t="n"/>
       <c r="AP181" s="15" t="n"/>
       <c r="AQ181" s="16" t="n"/>
+      <c r="AR181" s="16" t="n"/>
+      <c r="AS181" s="16" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="15" t="n"/>
@@ -10960,6 +11344,8 @@
       <c r="AO182" s="15" t="n"/>
       <c r="AP182" s="15" t="n"/>
       <c r="AQ182" s="16" t="n"/>
+      <c r="AR182" s="16" t="n"/>
+      <c r="AS182" s="16" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="15" t="n"/>
@@ -11013,6 +11399,8 @@
       <c r="AO183" s="15" t="n"/>
       <c r="AP183" s="15" t="n"/>
       <c r="AQ183" s="16" t="n"/>
+      <c r="AR183" s="16" t="n"/>
+      <c r="AS183" s="16" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="15" t="n"/>
@@ -11066,6 +11454,8 @@
       <c r="AO184" s="15" t="n"/>
       <c r="AP184" s="15" t="n"/>
       <c r="AQ184" s="16" t="n"/>
+      <c r="AR184" s="16" t="n"/>
+      <c r="AS184" s="16" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="15" t="n"/>
@@ -11119,6 +11509,8 @@
       <c r="AO185" s="15" t="n"/>
       <c r="AP185" s="15" t="n"/>
       <c r="AQ185" s="16" t="n"/>
+      <c r="AR185" s="16" t="n"/>
+      <c r="AS185" s="16" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="15" t="n"/>
@@ -11172,6 +11564,8 @@
       <c r="AO186" s="15" t="n"/>
       <c r="AP186" s="15" t="n"/>
       <c r="AQ186" s="16" t="n"/>
+      <c r="AR186" s="16" t="n"/>
+      <c r="AS186" s="16" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="15" t="n"/>
@@ -11225,6 +11619,8 @@
       <c r="AO187" s="15" t="n"/>
       <c r="AP187" s="15" t="n"/>
       <c r="AQ187" s="16" t="n"/>
+      <c r="AR187" s="16" t="n"/>
+      <c r="AS187" s="16" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="15" t="n"/>
@@ -11278,6 +11674,8 @@
       <c r="AO188" s="15" t="n"/>
       <c r="AP188" s="15" t="n"/>
       <c r="AQ188" s="16" t="n"/>
+      <c r="AR188" s="16" t="n"/>
+      <c r="AS188" s="16" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="15" t="n"/>
@@ -11331,6 +11729,8 @@
       <c r="AO189" s="15" t="n"/>
       <c r="AP189" s="15" t="n"/>
       <c r="AQ189" s="16" t="n"/>
+      <c r="AR189" s="16" t="n"/>
+      <c r="AS189" s="16" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="15" t="n"/>
@@ -11384,6 +11784,8 @@
       <c r="AO190" s="15" t="n"/>
       <c r="AP190" s="15" t="n"/>
       <c r="AQ190" s="16" t="n"/>
+      <c r="AR190" s="16" t="n"/>
+      <c r="AS190" s="16" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="15" t="n"/>
@@ -11437,6 +11839,8 @@
       <c r="AO191" s="15" t="n"/>
       <c r="AP191" s="15" t="n"/>
       <c r="AQ191" s="16" t="n"/>
+      <c r="AR191" s="16" t="n"/>
+      <c r="AS191" s="16" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="15" t="n"/>
@@ -11490,6 +11894,8 @@
       <c r="AO192" s="15" t="n"/>
       <c r="AP192" s="15" t="n"/>
       <c r="AQ192" s="16" t="n"/>
+      <c r="AR192" s="16" t="n"/>
+      <c r="AS192" s="16" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="15" t="n"/>
@@ -11543,6 +11949,8 @@
       <c r="AO193" s="15" t="n"/>
       <c r="AP193" s="15" t="n"/>
       <c r="AQ193" s="16" t="n"/>
+      <c r="AR193" s="16" t="n"/>
+      <c r="AS193" s="16" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="15" t="n"/>
@@ -11596,6 +12004,8 @@
       <c r="AO194" s="15" t="n"/>
       <c r="AP194" s="15" t="n"/>
       <c r="AQ194" s="16" t="n"/>
+      <c r="AR194" s="16" t="n"/>
+      <c r="AS194" s="16" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="15" t="n"/>
@@ -11649,6 +12059,8 @@
       <c r="AO195" s="15" t="n"/>
       <c r="AP195" s="15" t="n"/>
       <c r="AQ195" s="16" t="n"/>
+      <c r="AR195" s="16" t="n"/>
+      <c r="AS195" s="16" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="15" t="n"/>
@@ -11702,6 +12114,8 @@
       <c r="AO196" s="15" t="n"/>
       <c r="AP196" s="15" t="n"/>
       <c r="AQ196" s="16" t="n"/>
+      <c r="AR196" s="16" t="n"/>
+      <c r="AS196" s="16" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="15" t="n"/>
@@ -11755,6 +12169,8 @@
       <c r="AO197" s="15" t="n"/>
       <c r="AP197" s="15" t="n"/>
       <c r="AQ197" s="16" t="n"/>
+      <c r="AR197" s="16" t="n"/>
+      <c r="AS197" s="16" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="15" t="n"/>
@@ -11808,6 +12224,8 @@
       <c r="AO198" s="15" t="n"/>
       <c r="AP198" s="15" t="n"/>
       <c r="AQ198" s="16" t="n"/>
+      <c r="AR198" s="16" t="n"/>
+      <c r="AS198" s="16" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="15" t="n"/>
@@ -11861,6 +12279,8 @@
       <c r="AO199" s="15" t="n"/>
       <c r="AP199" s="15" t="n"/>
       <c r="AQ199" s="16" t="n"/>
+      <c r="AR199" s="16" t="n"/>
+      <c r="AS199" s="16" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="15" t="n"/>
@@ -11914,6 +12334,8 @@
       <c r="AO200" s="15" t="n"/>
       <c r="AP200" s="15" t="n"/>
       <c r="AQ200" s="16" t="n"/>
+      <c r="AR200" s="16" t="n"/>
+      <c r="AS200" s="16" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="15" t="n"/>
@@ -11967,6 +12389,8 @@
       <c r="AO201" s="15" t="n"/>
       <c r="AP201" s="15" t="n"/>
       <c r="AQ201" s="16" t="n"/>
+      <c r="AR201" s="16" t="n"/>
+      <c r="AS201" s="16" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="15" t="n"/>
@@ -12020,6 +12444,8 @@
       <c r="AO202" s="15" t="n"/>
       <c r="AP202" s="15" t="n"/>
       <c r="AQ202" s="16" t="n"/>
+      <c r="AR202" s="16" t="n"/>
+      <c r="AS202" s="16" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="15" t="n"/>
@@ -12073,6 +12499,8 @@
       <c r="AO203" s="15" t="n"/>
       <c r="AP203" s="15" t="n"/>
       <c r="AQ203" s="16" t="n"/>
+      <c r="AR203" s="16" t="n"/>
+      <c r="AS203" s="16" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="15" t="n"/>
@@ -12126,6 +12554,8 @@
       <c r="AO204" s="15" t="n"/>
       <c r="AP204" s="15" t="n"/>
       <c r="AQ204" s="16" t="n"/>
+      <c r="AR204" s="16" t="n"/>
+      <c r="AS204" s="16" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0" password="E84A"/>

</xml_diff>